<commit_message>
Corrections done on all files
</commit_message>
<xml_diff>
--- a/analyst/Franzi/rmonize/data_proc_elem/DPE_BGS98_FRANZI.xlsx
+++ b/analyst/Franzi/rmonize/data_proc_elem/DPE_BGS98_FRANZI.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\schwarz-f\Desktop\use-cases-harmonisation\analyst\Franzi\rmonize\data_proc_elem\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="K:\use-cases-harmonisation\use-cases-harmonisation\analyst\Franzi\rmonize\data_proc_elem\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{395728E3-4D76-44D9-A818-0EBB29684136}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F4ECCB5-CC0E-4E43-9131-C4DAB00508BB}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FA95D038-F567-4E66-BDED-85F5FC44E08E}"/>
   </bookViews>
@@ -214,7 +214,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -243,14 +243,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -272,16 +264,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -297,9 +288,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 – 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -337,7 +328,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 – 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -443,7 +434,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 – 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -585,7 +576,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -594,7 +585,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E14AF68-56D3-4388-ABCF-F9531188A834}">
   <dimension ref="A1:K14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="73.42578125" bestFit="1" customWidth="1"/>
@@ -861,10 +852,10 @@
       <c r="H10" t="s">
         <v>17</v>
       </c>
-      <c r="J10" s="5" t="s">
+      <c r="J10" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="K10" s="5" t="s">
+      <c r="K10" s="3" t="s">
         <v>54</v>
       </c>
     </row>
@@ -881,17 +872,17 @@
       <c r="F11" t="s">
         <v>59</v>
       </c>
-      <c r="G11" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="J11" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="K11" s="5" t="s">
-        <v>54</v>
+      <c r="G11" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J11" t="s">
+        <v>12</v>
+      </c>
+      <c r="K11" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>